<commit_message>
dados do painel — 14/09 13:32
</commit_message>
<xml_diff>
--- a/data/categorias.xlsx
+++ b/data/categorias.xlsx
@@ -564,7 +564,7 @@
         <v>202488.42</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>27.4</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="3">
@@ -1878,7 +1878,7 @@
         <v>51.5</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>26.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="16">

</xml_diff>